<commit_message>
added downloading feature for excel sheet
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -446,30 +446,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(-116, 39)</t>
+          <t>(78, 17)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(17, 11)</t>
+          <t>(78, 17)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>15262.00289263077</v>
+        <v>26.76330895578323</v>
       </c>
       <c r="D2" t="n">
-        <v>12672.78024010024</v>
+        <v>26.11678692319597</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Nevada, and Africa</t>
+          <t>telengana, and kukatpally</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(17, 11)</t>
+          <t>(78, 17)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -478,21 +478,21 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2076.091445540656</v>
+        <v>8802.629699685876</v>
       </c>
       <c r="D3" t="n">
-        <v>2058.837597875743</v>
+        <v>8602.315535096039</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Africa, and Tema</t>
+          <t>kukatpally, and Tema</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(-116, 39)</t>
+          <t>(78, 17)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -501,14 +501,14 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>13503.17437338391</v>
+        <v>8819.341941477658</v>
       </c>
       <c r="D4" t="n">
-        <v>11853.23509981646</v>
+        <v>8621.753207157857</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Nevada, and Tema</t>
+          <t>telengana, and Tema</t>
         </is>
       </c>
     </row>

</xml_diff>